<commit_message>
feat(saff-study): publish specification and test suite v1.4
</commit_message>
<xml_diff>
--- a/output/xlsx/LoginExtratorAdministrador--GT-.xlsx
+++ b/output/xlsx/LoginExtratorAdministrador--GT-.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="66">
   <si>
     <t xml:space="preserve">System: </t>
   </si>
@@ -101,7 +101,7 @@
     <t>SYSTEM exibe tela de login</t>
   </si>
   <si>
-    <t>administrador: digita o user e a password de um usuario administrador e pressiona o botao Login</t>
+    <t>administrador: digita o user e a password de um usuário administrador e pressiona o botao Login</t>
   </si>
   <si>
     <t>SYSTEM exibe tela de extracao por dispositivo</t>
@@ -110,16 +110,25 @@
     <t xml:space="preserve">Postcondition: </t>
   </si>
   <si>
+    <t>O usuario deve estar logado</t>
+  </si>
+  <si>
     <t>TC2</t>
   </si>
   <si>
     <t>Alternative Flow 1: User invalido</t>
   </si>
   <si>
-    <t>administrador: digita o user de um usuário invalido, digita uma password e pressiona o botao Login</t>
-  </si>
-  <si>
-    <t>SYSTEM exibe na pagina de login uma mensagem de usuario ou senha incorretos</t>
+    <t>administrador: digita o user de um usuário inválido, digita uma password e pressiona o botao Login</t>
+  </si>
+  <si>
+    <t>SYSTEM exibe mensagem “Invalid user or password” na tela de login</t>
+  </si>
+  <si>
+    <t>system: SYSTEM: exibe tela de login</t>
+  </si>
+  <si>
+    <t>exibe tela de login</t>
   </si>
   <si>
     <t>TC3</t>
@@ -131,7 +140,7 @@
     <t>administrador: digita o user de um usuário administrador corretamente, digita uma password invalida e pressiona o botao Login</t>
   </si>
   <si>
-    <t>SYSTEM abre um pop-up e exibe a mensagem de usuario ou senha incorretos; informa o numero de tentativas restantes ate que o usuario seja bloqueado</t>
+    <t>SYSTEM abre um pop-up e exibe a mensagem “User or Password incorrect. Attempts remaining until the account lockout: #tentativas restantes#” em um pop-up</t>
   </si>
   <si>
     <t>administrador: pressiona o botao Ok</t>
@@ -146,16 +155,16 @@
     <t>Alternative Flow 3: Numero de tentativas invalidas e 5</t>
   </si>
   <si>
-    <t>administrador: digita o user correte e o password invalido pela sexta vez e pressiona o botao Login</t>
-  </si>
-  <si>
-    <t>SYSTEM bloqueia o usuario e exibe uma mensagem informando que o usuario foi bloqueado</t>
+    <t>administrador: digita o user de um usuario administrador corretamente, digita uma password invalida pela sexta vez e pressiona o botao Login</t>
+  </si>
+  <si>
+    <t>SYSTEM bloqueia o usuário e exibe a mensagem 'This user has been blocked'</t>
   </si>
   <si>
     <t>administrador: tenta mais uma vez logar na conta do usuário, agora com dados validos</t>
   </si>
   <si>
-    <t>SYSTEM exibe mensagem informando usuario esta bloqueado</t>
+    <t>SYSTEM exibe mensagem informando usuario está bloqueado</t>
   </si>
   <si>
     <t>TC5</t>
@@ -179,7 +188,7 @@
     <t>TC6</t>
   </si>
   <si>
-    <t>Exception Flow 2: Sem conexao com o servidor e usuario nao deseja fazer extração offline</t>
+    <t>Exception Flow 2: Sem conexao com o servidor e usuário nao deseja fazer extração offline</t>
   </si>
   <si>
     <t>SYSTEM exibe pop-up questionando se o usuário deveja fazer extracoes offline</t>
@@ -194,7 +203,13 @@
     <t>Exception Flow 3: Usuario inativo por 90 dias</t>
   </si>
   <si>
-    <t>SYSTEM exibe mensagem indicando que usuario foi bloqueado</t>
+    <t>SYSTEM exibe a mensagem 'This user has been blocked'</t>
+  </si>
+  <si>
+    <t>administrador: executa programa externo que reinicia senha de super admin</t>
+  </si>
+  <si>
+    <t>SYSTEM processes action successfully</t>
   </si>
 </sst>
 </file>
@@ -286,13 +301,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="103.57421875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="115.1953125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="21.8984375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="124.36328125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="129.91796875" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="30.5234375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="17.578125" customWidth="true" bestFit="true"/>
   </cols>
@@ -434,7 +449,7 @@
         <v>31</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15">
@@ -442,7 +457,7 @@
         <v>11</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C15" t="s" s="1">
         <v>13</v>
@@ -456,7 +471,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E16" t="s" s="1">
         <v>17</v>
@@ -515,13 +530,13 @@
         <v>2.0</v>
       </c>
       <c r="B20" t="s" s="3">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C20" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D20" t="s" s="3">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E20" t="s" s="3">
         <v>27</v>
@@ -535,114 +550,114 @@
         <v>3.0</v>
       </c>
       <c r="B21" t="s" s="3">
+        <v>37</v>
+      </c>
+      <c r="C21" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D21" t="s" s="3">
+        <v>38</v>
+      </c>
+      <c r="E21" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F21" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="B22" t="s" s="3">
         <v>29</v>
       </c>
-      <c r="C21" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D21" t="s" s="3">
+      <c r="C22" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D22" t="s" s="3">
         <v>30</v>
       </c>
-      <c r="E21" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F21" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s" s="1">
+      <c r="E22" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F22" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="1">
         <v>31</v>
       </c>
-      <c r="B22" t="s" s="0">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B25" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="C25" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E25" t="s" s="1">
-        <v>14</v>
+      <c r="B23" t="s" s="0">
+        <v>32</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="1">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>37</v>
+        <v>39</v>
+      </c>
+      <c r="C26" t="s" s="1">
+        <v>13</v>
       </c>
       <c r="E26" t="s" s="1">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E27" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B27" t="s" s="0">
+      <c r="B28" t="s" s="0">
         <v>19</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="s" s="2">
+    <row r="29">
+      <c r="A29" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B28" t="s" s="2">
+      <c r="B29" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="C28" t="s" s="2">
+      <c r="C29" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D28" t="s" s="2">
+      <c r="D29" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="E28" t="s" s="2">
+      <c r="E29" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="F28" t="s" s="2">
+      <c r="F29" t="s" s="2">
         <v>25</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B29" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C29" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D29" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E29" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F29" t="s" s="3">
-        <v>27</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n" s="4">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B30" t="s" s="3">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C30" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D30" t="s" s="3">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="E30" t="s" s="3">
         <v>27</v>
@@ -653,16 +668,16 @@
     </row>
     <row r="31">
       <c r="A31" t="n" s="4">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="B31" t="s" s="3">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C31" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D31" t="s" s="3">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E31" t="s" s="3">
         <v>27</v>
@@ -673,494 +688,554 @@
     </row>
     <row r="32">
       <c r="A32" t="n" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="B32" t="s" s="3">
+        <v>43</v>
+      </c>
+      <c r="C32" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D32" t="s" s="3">
+        <v>44</v>
+      </c>
+      <c r="E32" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F32" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n" s="4">
         <v>4.0</v>
       </c>
-      <c r="B32" t="s" s="3">
+      <c r="B33" t="s" s="3">
+        <v>37</v>
+      </c>
+      <c r="C33" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D33" t="s" s="3">
+        <v>38</v>
+      </c>
+      <c r="E33" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F33" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="B34" t="s" s="3">
         <v>29</v>
       </c>
-      <c r="C32" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D32" t="s" s="3">
+      <c r="C34" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D34" t="s" s="3">
         <v>30</v>
       </c>
-      <c r="E32" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F32" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="s" s="1">
+      <c r="E34" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F34" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="1">
         <v>31</v>
       </c>
-      <c r="B33" t="s" s="0">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B36" t="s" s="0">
-        <v>42</v>
-      </c>
-      <c r="C36" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E36" t="s" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B37" t="s" s="0">
-        <v>43</v>
-      </c>
-      <c r="E37" t="s" s="1">
-        <v>17</v>
+      <c r="B35" t="s" s="0">
+        <v>32</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C38" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E38" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="E39" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B38" t="s" s="0">
+      <c r="B40" t="s" s="0">
         <v>19</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="s" s="2">
+    <row r="41">
+      <c r="A41" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B39" t="s" s="2">
+      <c r="B41" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="C39" t="s" s="2">
+      <c r="C41" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D39" t="s" s="2">
+      <c r="D41" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="E39" t="s" s="2">
+      <c r="E41" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="F39" t="s" s="2">
+      <c r="F41" t="s" s="2">
         <v>25</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B40" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C40" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D40" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E40" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F40" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="B41" t="s" s="3">
-        <v>44</v>
-      </c>
-      <c r="C41" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D41" t="s" s="3">
-        <v>45</v>
-      </c>
-      <c r="E41" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F41" t="s" s="3">
-        <v>27</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B42" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C42" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D42" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E42" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F42" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B43" t="s" s="3">
+        <v>47</v>
+      </c>
+      <c r="C43" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D43" t="s" s="3">
+        <v>48</v>
+      </c>
+      <c r="E43" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F43" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n" s="4">
         <v>3.0</v>
       </c>
-      <c r="B42" t="s" s="3">
-        <v>46</v>
-      </c>
-      <c r="C42" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D42" t="s" s="3">
-        <v>47</v>
-      </c>
-      <c r="E42" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F42" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="s" s="1">
+      <c r="B44" t="s" s="3">
+        <v>49</v>
+      </c>
+      <c r="C44" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D44" t="s" s="3">
+        <v>50</v>
+      </c>
+      <c r="E44" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F44" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s" s="1">
         <v>31</v>
       </c>
-      <c r="B43" t="s" s="0">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B46" t="s" s="0">
-        <v>48</v>
-      </c>
-      <c r="C46" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E46" t="s" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B47" t="s" s="0">
-        <v>49</v>
-      </c>
-      <c r="E47" t="s" s="1">
-        <v>17</v>
+      <c r="B45" t="s" s="0">
+        <v>32</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B48" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="C48" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E48" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B49" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E49" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B48" t="s" s="0">
+      <c r="B50" t="s" s="0">
         <v>19</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="s" s="2">
+    <row r="51">
+      <c r="A51" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B49" t="s" s="2">
+      <c r="B51" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="C49" t="s" s="2">
+      <c r="C51" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D49" t="s" s="2">
+      <c r="D51" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="E49" t="s" s="2">
+      <c r="E51" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="F49" t="s" s="2">
+      <c r="F51" t="s" s="2">
         <v>25</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B50" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C50" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D50" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E50" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F50" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="B51" t="s" s="3">
-        <v>29</v>
-      </c>
-      <c r="C51" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D51" t="s" s="3">
-        <v>50</v>
-      </c>
-      <c r="E51" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F51" t="s" s="3">
-        <v>27</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B52" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C52" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D52" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E52" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F52" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B53" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C53" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D53" t="s" s="3">
+        <v>53</v>
+      </c>
+      <c r="E53" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F53" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n" s="4">
         <v>3.0</v>
       </c>
-      <c r="B52" t="s" s="3">
-        <v>51</v>
-      </c>
-      <c r="C52" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D52" t="s" s="3">
-        <v>52</v>
-      </c>
-      <c r="E52" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F52" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="s" s="1">
+      <c r="B54" t="s" s="3">
+        <v>54</v>
+      </c>
+      <c r="C54" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D54" t="s" s="3">
+        <v>55</v>
+      </c>
+      <c r="E54" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F54" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="1">
         <v>31</v>
       </c>
-      <c r="B53" t="s" s="0">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B56" t="s" s="0">
-        <v>54</v>
-      </c>
-      <c r="C56" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E56" t="s" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B57" t="s" s="0">
-        <v>55</v>
-      </c>
-      <c r="E57" t="s" s="1">
-        <v>17</v>
+      <c r="B55" t="s" s="0">
+        <v>56</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B58" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="C58" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E58" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B59" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="E59" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B58" t="s" s="0">
+      <c r="B60" t="s" s="0">
         <v>19</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="s" s="2">
+    <row r="61">
+      <c r="A61" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B59" t="s" s="2">
+      <c r="B61" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="C59" t="s" s="2">
+      <c r="C61" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D59" t="s" s="2">
+      <c r="D61" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="E59" t="s" s="2">
+      <c r="E61" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="F59" t="s" s="2">
+      <c r="F61" t="s" s="2">
         <v>25</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B60" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C60" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D60" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E60" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F60" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="n" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="B61" t="s" s="3">
-        <v>29</v>
-      </c>
-      <c r="C61" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D61" t="s" s="3">
-        <v>56</v>
-      </c>
-      <c r="E61" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F61" t="s" s="3">
-        <v>27</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B62" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C62" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D62" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E62" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F62" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B63" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C63" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D63" t="s" s="3">
+        <v>59</v>
+      </c>
+      <c r="E63" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F63" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n" s="4">
         <v>3.0</v>
       </c>
-      <c r="B62" t="s" s="3">
-        <v>57</v>
-      </c>
-      <c r="C62" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D62" t="s" s="3">
-        <v>41</v>
-      </c>
-      <c r="E62" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F62" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="s" s="1">
+      <c r="B64" t="s" s="3">
+        <v>60</v>
+      </c>
+      <c r="C64" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D64" t="s" s="3">
+        <v>44</v>
+      </c>
+      <c r="E64" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F64" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s" s="1">
         <v>31</v>
       </c>
-      <c r="B63" t="s" s="0">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B66" t="s" s="0">
-        <v>58</v>
-      </c>
-      <c r="C66" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E66" t="s" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B67" t="s" s="0">
-        <v>59</v>
-      </c>
-      <c r="E67" t="s" s="1">
-        <v>17</v>
+      <c r="B65" t="s" s="0">
+        <v>56</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B68" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="C68" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E68" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B69" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="E69" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s" s="1">
         <v>18</v>
       </c>
-      <c r="B68" t="s" s="0">
+      <c r="B70" t="s" s="0">
         <v>19</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="s" s="2">
+    <row r="71">
+      <c r="A71" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B69" t="s" s="2">
+      <c r="B71" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="C69" t="s" s="2">
+      <c r="C71" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D69" t="s" s="2">
+      <c r="D71" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="E69" t="s" s="2">
+      <c r="E71" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="F69" t="s" s="2">
+      <c r="F71" t="s" s="2">
         <v>25</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="n" s="4">
+    <row r="72">
+      <c r="A72" t="n" s="4">
         <v>1.0</v>
       </c>
-      <c r="B70" t="s" s="3">
+      <c r="B72" t="s" s="3">
         <v>26</v>
       </c>
-      <c r="C70" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D70" t="s" s="3">
+      <c r="C72" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D72" t="s" s="3">
         <v>28</v>
       </c>
-      <c r="E70" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F70" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="n" s="4">
+      <c r="E72" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F72" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n" s="4">
         <v>2.0</v>
       </c>
-      <c r="B71" t="s" s="3">
+      <c r="B73" t="s" s="3">
         <v>29</v>
       </c>
-      <c r="C71" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D71" t="s" s="3">
-        <v>60</v>
-      </c>
-      <c r="E71" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F71" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="s" s="1">
+      <c r="C73" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D73" t="s" s="3">
+        <v>63</v>
+      </c>
+      <c r="E73" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F73" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="B74" t="s" s="3">
+        <v>64</v>
+      </c>
+      <c r="C74" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D74" t="s" s="3">
+        <v>65</v>
+      </c>
+      <c r="E74" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F74" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s" s="1">
         <v>31</v>
       </c>
-      <c r="B72" t="s" s="0">
-        <v>53</v>
+      <c r="B75" t="s" s="0">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>